<commit_message>
feat(caras): merge cells D16:E16 for Tamaño Máximo Nominal in template
</commit_message>
<xml_diff>
--- a/app/templates/informes/Informes agregado/CARAS/Template_Caras.xlsx
+++ b/app/templates/informes/Informes agregado/CARAS/Template_Caras.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Mi unidad\3.0 Formatos e informes\2026\1.0 Informe de ensayo\1.2 Informe agregados\INFORME ACREDITADO-E ISO\1.1 JUNIO 15-06-26\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\informes\Informes agregado\CARAS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{932A941E-D8D6-44C1-B630-312168C6A384}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6735CA2A-E7C1-4F26-A400-37BC3DBE8C10}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FORMATO" sheetId="96" r:id="rId1"/>
@@ -3693,9 +3693,6 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="3" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="43" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="43" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -3875,45 +3872,39 @@
     <xf numFmtId="0" fontId="6" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="179" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3928,6 +3919,12 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="5" quotePrefix="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
@@ -4131,6 +4128,9 @@
     </xf>
     <xf numFmtId="176" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="8">
@@ -4399,7 +4399,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4435,7 +4435,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4473,7 +4473,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -4650,7 +4650,7 @@
                 <a:cs typeface="Arial"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145561856"/>
@@ -4686,7 +4686,7 @@
                 <a:cs typeface="Calibri"/>
               </a:defRPr>
             </a:pPr>
-            <a:endParaRPr lang="es-ES"/>
+            <a:endParaRPr lang="es-PE"/>
           </a:p>
         </c:txPr>
         <c:crossAx val="145560320"/>
@@ -4724,7 +4724,7 @@
           <a:cs typeface="Calibri"/>
         </a:defRPr>
       </a:pPr>
-      <a:endParaRPr lang="es-ES"/>
+      <a:endParaRPr lang="es-PE"/>
     </a:p>
   </c:txPr>
   <c:printSettings>
@@ -5947,7 +5947,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6006,7 +6006,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6081,7 +6081,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink3.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="-------"/>
@@ -6156,7 +6156,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink4.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="BGA"/>
@@ -7191,13 +7191,13 @@
     <row r="2" spans="2:11" ht="12" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="341"/>
       <c r="C2" s="342"/>
-      <c r="D2" s="444" t="s">
+      <c r="D2" s="443" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="444"/>
-      <c r="F2" s="444"/>
-      <c r="G2" s="444"/>
-      <c r="H2" s="445"/>
+      <c r="E2" s="443"/>
+      <c r="F2" s="443"/>
+      <c r="G2" s="443"/>
+      <c r="H2" s="444"/>
       <c r="J2" s="418" t="s">
         <v>195</v>
       </c>
@@ -7206,13 +7206,13 @@
     <row r="3" spans="2:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="341"/>
       <c r="C3" s="342"/>
-      <c r="D3" s="446" t="s">
+      <c r="D3" s="445" t="s">
         <v>154</v>
       </c>
-      <c r="E3" s="446"/>
-      <c r="F3" s="446"/>
-      <c r="G3" s="446"/>
-      <c r="H3" s="447"/>
+      <c r="E3" s="445"/>
+      <c r="F3" s="445"/>
+      <c r="G3" s="445"/>
+      <c r="H3" s="446"/>
       <c r="J3" s="418" t="s">
         <v>196</v>
       </c>
@@ -7263,10 +7263,10 @@
       <c r="D7" s="350" t="s">
         <v>156</v>
       </c>
-      <c r="E7" s="448" t="s">
+      <c r="E7" s="447" t="s">
         <v>157</v>
       </c>
-      <c r="F7" s="448"/>
+      <c r="F7" s="447"/>
       <c r="G7" s="350" t="s">
         <v>158</v>
       </c>
@@ -7280,8 +7280,8 @@
       <c r="B8" s="351"/>
       <c r="C8" s="352"/>
       <c r="D8" s="353"/>
-      <c r="E8" s="449"/>
-      <c r="F8" s="449"/>
+      <c r="E8" s="448"/>
+      <c r="F8" s="448"/>
       <c r="G8" s="353"/>
       <c r="H8" s="343"/>
       <c r="J8" s="418" t="s">
@@ -7291,8 +7291,8 @@
     </row>
     <row r="9" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="351"/>
-      <c r="C9" s="450"/>
-      <c r="D9" s="450"/>
+      <c r="C9" s="449"/>
+      <c r="D9" s="449"/>
       <c r="E9" s="354"/>
       <c r="F9" s="354"/>
       <c r="G9" s="354"/>
@@ -7314,30 +7314,30 @@
       <c r="K10" s="422"/>
     </row>
     <row r="11" spans="2:11" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="441" t="s">
+      <c r="B11" s="440" t="s">
         <v>159</v>
       </c>
-      <c r="C11" s="442"/>
-      <c r="D11" s="442"/>
-      <c r="E11" s="442"/>
-      <c r="F11" s="442"/>
-      <c r="G11" s="442"/>
-      <c r="H11" s="443"/>
+      <c r="C11" s="441"/>
+      <c r="D11" s="441"/>
+      <c r="E11" s="441"/>
+      <c r="F11" s="441"/>
+      <c r="G11" s="441"/>
+      <c r="H11" s="442"/>
       <c r="J11" s="418" t="s">
         <v>82</v>
       </c>
       <c r="K11" s="422"/>
     </row>
     <row r="12" spans="2:11" ht="13.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B12" s="451" t="s">
+      <c r="B12" s="450" t="s">
         <v>160</v>
       </c>
-      <c r="C12" s="452"/>
-      <c r="D12" s="452"/>
-      <c r="E12" s="452"/>
-      <c r="F12" s="452"/>
-      <c r="G12" s="452"/>
-      <c r="H12" s="453"/>
+      <c r="C12" s="451"/>
+      <c r="D12" s="451"/>
+      <c r="E12" s="451"/>
+      <c r="F12" s="451"/>
+      <c r="G12" s="451"/>
+      <c r="H12" s="452"/>
       <c r="J12" s="418" t="s">
         <v>83</v>
       </c>
@@ -7362,18 +7362,18 @@
       <c r="C14" s="360"/>
       <c r="D14" s="361"/>
       <c r="E14" s="362"/>
-      <c r="G14" s="454" t="s">
+      <c r="G14" s="453" t="s">
         <v>162</v>
       </c>
-      <c r="H14" s="455"/>
+      <c r="H14" s="454"/>
       <c r="J14" s="421"/>
       <c r="K14" s="422"/>
     </row>
     <row r="15" spans="2:11" ht="24" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="456" t="s">
+      <c r="B15" s="455" t="s">
         <v>163</v>
       </c>
-      <c r="C15" s="457"/>
+      <c r="C15" s="456"/>
       <c r="D15" s="290" t="s">
         <v>204</v>
       </c>
@@ -7396,8 +7396,8 @@
         <v>68</v>
       </c>
       <c r="C16" s="366"/>
-      <c r="D16" s="426"/>
-      <c r="E16" s="427"/>
+      <c r="D16" s="556"/>
+      <c r="E16" s="426"/>
       <c r="G16" s="367" t="s">
         <v>167</v>
       </c>
@@ -7414,8 +7414,8 @@
         <v>168</v>
       </c>
       <c r="C17" s="290"/>
-      <c r="D17" s="458"/>
-      <c r="E17" s="459"/>
+      <c r="D17" s="457"/>
+      <c r="E17" s="458"/>
       <c r="G17" s="367" t="s">
         <v>169</v>
       </c>
@@ -7438,10 +7438,10 @@
       <c r="E18" s="371" t="s">
         <v>172</v>
       </c>
-      <c r="G18" s="460" t="s">
+      <c r="G18" s="459" t="s">
         <v>173</v>
       </c>
-      <c r="H18" s="460"/>
+      <c r="H18" s="459"/>
     </row>
     <row r="19" spans="2:14" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="372" t="s">
@@ -7451,8 +7451,8 @@
       <c r="D19" s="374"/>
       <c r="E19" s="375"/>
       <c r="F19" s="376"/>
-      <c r="G19" s="461"/>
-      <c r="H19" s="461"/>
+      <c r="G19" s="460"/>
+      <c r="H19" s="460"/>
     </row>
     <row r="20" spans="2:14" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="368" t="s">
@@ -7460,7 +7460,7 @@
       </c>
       <c r="C20" s="373"/>
       <c r="D20" s="377"/>
-      <c r="E20" s="428"/>
+      <c r="E20" s="427"/>
       <c r="F20" s="376"/>
       <c r="G20" s="378"/>
       <c r="H20" s="379"/>
@@ -7471,7 +7471,7 @@
       </c>
       <c r="C21" s="324"/>
       <c r="D21" s="13"/>
-      <c r="E21" s="429"/>
+      <c r="E21" s="428"/>
       <c r="F21" s="376"/>
       <c r="G21" s="13"/>
       <c r="H21" s="13"/>
@@ -7482,7 +7482,7 @@
       </c>
       <c r="C22" s="382"/>
       <c r="D22" s="383"/>
-      <c r="E22" s="429"/>
+      <c r="E22" s="428"/>
       <c r="F22" s="20" t="s">
         <v>177</v>
       </c>
@@ -7493,7 +7493,7 @@
         <v>112</v>
       </c>
       <c r="C23" s="385"/>
-      <c r="E23" s="429"/>
+      <c r="E23" s="428"/>
       <c r="F23" s="386"/>
       <c r="G23" s="16"/>
       <c r="H23" s="16"/>
@@ -7504,7 +7504,7 @@
       </c>
       <c r="C24" s="387"/>
       <c r="D24" s="388"/>
-      <c r="E24" s="429"/>
+      <c r="E24" s="428"/>
       <c r="F24" s="15"/>
       <c r="G24" s="16"/>
       <c r="H24" s="16"/>
@@ -7514,7 +7514,7 @@
         <v>178</v>
       </c>
       <c r="C25" s="385"/>
-      <c r="E25" s="430"/>
+      <c r="E25" s="429"/>
       <c r="F25" s="15"/>
       <c r="G25" s="16"/>
       <c r="H25" s="16"/>
@@ -7539,57 +7539,57 @@
       <c r="H27" s="16"/>
     </row>
     <row r="28" spans="2:14" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B28" s="464" t="s">
+      <c r="B28" s="463" t="s">
         <v>181</v>
       </c>
-      <c r="C28" s="464"/>
-      <c r="D28" s="464"/>
-      <c r="E28" s="464"/>
-      <c r="F28" s="464"/>
-      <c r="G28" s="464"/>
-      <c r="H28" s="464"/>
+      <c r="C28" s="463"/>
+      <c r="D28" s="463"/>
+      <c r="E28" s="463"/>
+      <c r="F28" s="463"/>
+      <c r="G28" s="463"/>
+      <c r="H28" s="463"/>
       <c r="L28" s="392"/>
       <c r="M28" s="392"/>
       <c r="N28" s="392"/>
     </row>
     <row r="29" spans="2:14" ht="24.6" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B29" s="465" t="s">
+      <c r="B29" s="464" t="s">
         <v>182</v>
       </c>
-      <c r="C29" s="465"/>
-      <c r="D29" s="465"/>
-      <c r="E29" s="465"/>
-      <c r="F29" s="465"/>
-      <c r="G29" s="465"/>
-      <c r="H29" s="465"/>
+      <c r="C29" s="464"/>
+      <c r="D29" s="464"/>
+      <c r="E29" s="464"/>
+      <c r="F29" s="464"/>
+      <c r="G29" s="464"/>
+      <c r="H29" s="464"/>
       <c r="L29" s="392"/>
       <c r="M29" s="392"/>
       <c r="N29" s="392"/>
     </row>
     <row r="30" spans="2:14" ht="16.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B30" s="466" t="s">
+      <c r="B30" s="465" t="s">
         <v>183</v>
       </c>
-      <c r="C30" s="466"/>
-      <c r="D30" s="466"/>
-      <c r="E30" s="466"/>
-      <c r="F30" s="466"/>
-      <c r="G30" s="466"/>
-      <c r="H30" s="466"/>
+      <c r="C30" s="465"/>
+      <c r="D30" s="465"/>
+      <c r="E30" s="465"/>
+      <c r="F30" s="465"/>
+      <c r="G30" s="465"/>
+      <c r="H30" s="465"/>
       <c r="L30" s="392"/>
       <c r="M30" s="392"/>
       <c r="N30" s="392"/>
     </row>
     <row r="31" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B31" s="467" t="s">
+      <c r="B31" s="466" t="s">
         <v>184</v>
       </c>
-      <c r="C31" s="468"/>
-      <c r="D31" s="469"/>
-      <c r="E31" s="473" t="s">
+      <c r="C31" s="467"/>
+      <c r="D31" s="468"/>
+      <c r="E31" s="472" t="s">
         <v>185</v>
       </c>
-      <c r="F31" s="473"/>
+      <c r="F31" s="472"/>
       <c r="G31" s="393" t="s">
         <v>186</v>
       </c>
@@ -7598,13 +7598,13 @@
       <c r="N31" s="392"/>
     </row>
     <row r="32" spans="2:14" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B32" s="470"/>
-      <c r="C32" s="471"/>
-      <c r="D32" s="472"/>
-      <c r="E32" s="474" t="s">
+      <c r="B32" s="469"/>
+      <c r="C32" s="470"/>
+      <c r="D32" s="471"/>
+      <c r="E32" s="473" t="s">
         <v>187</v>
       </c>
-      <c r="F32" s="475"/>
+      <c r="F32" s="474"/>
       <c r="G32" s="394" t="s">
         <v>187</v>
       </c>
@@ -7621,8 +7621,8 @@
       </c>
       <c r="C33" s="396"/>
       <c r="D33" s="397"/>
-      <c r="E33" s="462"/>
-      <c r="F33" s="463"/>
+      <c r="E33" s="461"/>
+      <c r="F33" s="462"/>
       <c r="G33" s="398"/>
     </row>
     <row r="34" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7634,8 +7634,8 @@
       </c>
       <c r="C34" s="399"/>
       <c r="D34" s="377"/>
-      <c r="E34" s="462"/>
-      <c r="F34" s="463"/>
+      <c r="E34" s="461"/>
+      <c r="F34" s="462"/>
       <c r="G34" s="398"/>
     </row>
     <row r="35" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7647,18 +7647,18 @@
       </c>
       <c r="C35" s="399"/>
       <c r="D35" s="377"/>
-      <c r="E35" s="462"/>
-      <c r="F35" s="463"/>
+      <c r="E35" s="461"/>
+      <c r="F35" s="462"/>
       <c r="G35" s="244"/>
     </row>
     <row r="36" spans="1:8" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B36" s="395"/>
       <c r="C36" s="399"/>
       <c r="D36" s="377"/>
-      <c r="E36" s="474" t="s">
+      <c r="E36" s="473" t="s">
         <v>188</v>
       </c>
-      <c r="F36" s="475"/>
+      <c r="F36" s="474"/>
       <c r="G36" s="394" t="s">
         <v>188</v>
       </c>
@@ -7669,8 +7669,8 @@
       </c>
       <c r="C37" s="399"/>
       <c r="D37" s="377"/>
-      <c r="E37" s="462"/>
-      <c r="F37" s="463"/>
+      <c r="E37" s="461"/>
+      <c r="F37" s="462"/>
       <c r="G37" s="244"/>
     </row>
     <row r="38" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7682,8 +7682,8 @@
       </c>
       <c r="C38" s="399"/>
       <c r="D38" s="377"/>
-      <c r="E38" s="462"/>
-      <c r="F38" s="463"/>
+      <c r="E38" s="461"/>
+      <c r="F38" s="462"/>
       <c r="G38" s="244"/>
     </row>
     <row r="39" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7695,8 +7695,8 @@
       </c>
       <c r="C39" s="399"/>
       <c r="D39" s="377"/>
-      <c r="E39" s="462"/>
-      <c r="F39" s="463"/>
+      <c r="E39" s="461"/>
+      <c r="F39" s="462"/>
       <c r="G39" s="244"/>
     </row>
     <row r="40" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7708,8 +7708,8 @@
       </c>
       <c r="C40" s="402"/>
       <c r="D40" s="403"/>
-      <c r="E40" s="476"/>
-      <c r="F40" s="477"/>
+      <c r="E40" s="475"/>
+      <c r="F40" s="476"/>
       <c r="G40" s="404"/>
     </row>
     <row r="41" spans="1:8" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.25">
@@ -7718,8 +7718,8 @@
       </c>
       <c r="C41" s="399"/>
       <c r="D41" s="377"/>
-      <c r="E41" s="478"/>
-      <c r="F41" s="478"/>
+      <c r="E41" s="477"/>
+      <c r="F41" s="477"/>
       <c r="G41" s="405"/>
     </row>
     <row r="42" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
@@ -7787,20 +7787,20 @@
       <c r="B49" s="417" t="s">
         <v>147</v>
       </c>
-      <c r="E49" s="479"/>
-      <c r="F49" s="479"/>
+      <c r="E49" s="478"/>
+      <c r="F49" s="478"/>
     </row>
     <row r="50" spans="2:8" ht="7.2" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="51" spans="2:8" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B51" s="480" t="s">
+      <c r="B51" s="479" t="s">
         <v>194</v>
       </c>
-      <c r="C51" s="480"/>
-      <c r="D51" s="480"/>
-      <c r="E51" s="480"/>
-      <c r="F51" s="480"/>
-      <c r="G51" s="480"/>
-      <c r="H51" s="480"/>
+      <c r="C51" s="479"/>
+      <c r="D51" s="479"/>
+      <c r="E51" s="479"/>
+      <c r="F51" s="479"/>
+      <c r="G51" s="479"/>
+      <c r="H51" s="479"/>
     </row>
   </sheetData>
   <protectedRanges>
@@ -7880,36 +7880,36 @@
       <c r="M1" s="126"/>
     </row>
     <row r="2" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="484" t="s">
+      <c r="A2" s="480" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="484"/>
-      <c r="C2" s="484"/>
-      <c r="D2" s="484"/>
-      <c r="E2" s="484"/>
-      <c r="F2" s="484"/>
-      <c r="G2" s="484"/>
-      <c r="H2" s="484"/>
-      <c r="I2" s="484"/>
-      <c r="J2" s="484"/>
-      <c r="K2" s="484"/>
+      <c r="B2" s="480"/>
+      <c r="C2" s="480"/>
+      <c r="D2" s="480"/>
+      <c r="E2" s="480"/>
+      <c r="F2" s="480"/>
+      <c r="G2" s="480"/>
+      <c r="H2" s="480"/>
+      <c r="I2" s="480"/>
+      <c r="J2" s="480"/>
+      <c r="K2" s="480"/>
       <c r="L2" s="128"/>
       <c r="M2" s="128"/>
     </row>
     <row r="3" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="485">
-        <v>0</v>
-      </c>
-      <c r="B3" s="485"/>
-      <c r="C3" s="485"/>
-      <c r="D3" s="485"/>
-      <c r="E3" s="485"/>
-      <c r="F3" s="485"/>
-      <c r="G3" s="485"/>
-      <c r="H3" s="485"/>
-      <c r="I3" s="485"/>
-      <c r="J3" s="485"/>
-      <c r="K3" s="485"/>
+      <c r="A3" s="481">
+        <v>0</v>
+      </c>
+      <c r="B3" s="481"/>
+      <c r="C3" s="481"/>
+      <c r="D3" s="481"/>
+      <c r="E3" s="481"/>
+      <c r="F3" s="481"/>
+      <c r="G3" s="481"/>
+      <c r="H3" s="481"/>
+      <c r="I3" s="481"/>
+      <c r="J3" s="481"/>
+      <c r="K3" s="481"/>
       <c r="L3" s="129"/>
       <c r="M3" s="129"/>
     </row>
@@ -7933,15 +7933,15 @@
       <c r="B5" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C5" s="495">
+      <c r="C5" s="492">
         <f>+FORMATO!K2</f>
         <v>0</v>
       </c>
-      <c r="D5" s="495"/>
-      <c r="E5" s="495"/>
-      <c r="F5" s="495"/>
-      <c r="G5" s="495"/>
-      <c r="H5" s="495"/>
+      <c r="D5" s="492"/>
+      <c r="E5" s="492"/>
+      <c r="F5" s="492"/>
+      <c r="G5" s="492"/>
+      <c r="H5" s="492"/>
       <c r="I5" s="7" t="s">
         <v>78</v>
       </c>
@@ -7959,15 +7959,15 @@
       <c r="B6" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C6" s="495">
+      <c r="C6" s="492">
         <f>+FORMATO!K3</f>
         <v>0</v>
       </c>
-      <c r="D6" s="495"/>
-      <c r="E6" s="495"/>
-      <c r="F6" s="495"/>
-      <c r="G6" s="495"/>
-      <c r="H6" s="495"/>
+      <c r="D6" s="492"/>
+      <c r="E6" s="492"/>
+      <c r="F6" s="492"/>
+      <c r="G6" s="492"/>
+      <c r="H6" s="492"/>
       <c r="I6" s="8" t="s">
         <v>79</v>
       </c>
@@ -7986,15 +7986,15 @@
       <c r="B7" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="495">
+      <c r="C7" s="492">
         <f>+FORMATO!K4</f>
         <v>0</v>
       </c>
-      <c r="D7" s="495"/>
-      <c r="E7" s="495"/>
-      <c r="F7" s="495"/>
-      <c r="G7" s="495"/>
-      <c r="H7" s="495"/>
+      <c r="D7" s="492"/>
+      <c r="E7" s="492"/>
+      <c r="F7" s="492"/>
+      <c r="G7" s="492"/>
+      <c r="H7" s="492"/>
       <c r="I7" s="8" t="s">
         <v>81</v>
       </c>
@@ -8014,16 +8014,16 @@
       <c r="B8" s="148" t="s">
         <v>69</v>
       </c>
-      <c r="C8" s="495">
+      <c r="C8" s="492">
         <f>+FORMATO!K5</f>
         <v>0</v>
       </c>
-      <c r="D8" s="495"/>
-      <c r="E8" s="495"/>
-      <c r="F8" s="495"/>
-      <c r="G8" s="495"/>
-      <c r="H8" s="495"/>
-      <c r="I8" s="431" t="s">
+      <c r="D8" s="492"/>
+      <c r="E8" s="492"/>
+      <c r="F8" s="492"/>
+      <c r="G8" s="492"/>
+      <c r="H8" s="492"/>
+      <c r="I8" s="430" t="s">
         <v>80</v>
       </c>
       <c r="J8" s="149" t="s">
@@ -8064,36 +8064,36 @@
       <c r="K10" s="4"/>
     </row>
     <row r="11" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="486" t="s">
+      <c r="A11" s="482" t="s">
         <v>144</v>
       </c>
-      <c r="B11" s="487"/>
-      <c r="C11" s="487"/>
-      <c r="D11" s="487"/>
-      <c r="E11" s="487"/>
-      <c r="F11" s="487"/>
-      <c r="G11" s="487"/>
-      <c r="H11" s="487"/>
-      <c r="I11" s="487"/>
-      <c r="J11" s="487"/>
-      <c r="K11" s="488"/>
+      <c r="B11" s="483"/>
+      <c r="C11" s="483"/>
+      <c r="D11" s="483"/>
+      <c r="E11" s="483"/>
+      <c r="F11" s="483"/>
+      <c r="G11" s="483"/>
+      <c r="H11" s="483"/>
+      <c r="I11" s="483"/>
+      <c r="J11" s="483"/>
+      <c r="K11" s="484"/>
       <c r="L11" s="131"/>
       <c r="M11" s="131"/>
     </row>
     <row r="12" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="489" t="s">
+      <c r="A12" s="485" t="s">
         <v>146</v>
       </c>
-      <c r="B12" s="490"/>
-      <c r="C12" s="490"/>
-      <c r="D12" s="490"/>
-      <c r="E12" s="490"/>
-      <c r="F12" s="490"/>
-      <c r="G12" s="490"/>
-      <c r="H12" s="490"/>
-      <c r="I12" s="490"/>
-      <c r="J12" s="490"/>
-      <c r="K12" s="491"/>
+      <c r="B12" s="486"/>
+      <c r="C12" s="486"/>
+      <c r="D12" s="486"/>
+      <c r="E12" s="486"/>
+      <c r="F12" s="486"/>
+      <c r="G12" s="486"/>
+      <c r="H12" s="486"/>
+      <c r="I12" s="486"/>
+      <c r="J12" s="486"/>
+      <c r="K12" s="487"/>
       <c r="L12" s="131"/>
       <c r="M12" s="136"/>
     </row>
@@ -8245,19 +8245,19 @@
       <c r="M19" s="126"/>
     </row>
     <row r="20" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="492" t="s">
+      <c r="A20" s="489" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="493"/>
-      <c r="C20" s="493"/>
-      <c r="D20" s="493"/>
-      <c r="E20" s="493"/>
-      <c r="F20" s="493"/>
-      <c r="G20" s="493"/>
-      <c r="H20" s="493"/>
-      <c r="I20" s="493"/>
-      <c r="J20" s="493"/>
-      <c r="K20" s="494"/>
+      <c r="B20" s="490"/>
+      <c r="C20" s="490"/>
+      <c r="D20" s="490"/>
+      <c r="E20" s="490"/>
+      <c r="F20" s="490"/>
+      <c r="G20" s="490"/>
+      <c r="H20" s="490"/>
+      <c r="I20" s="490"/>
+      <c r="J20" s="490"/>
+      <c r="K20" s="491"/>
       <c r="L20" s="20"/>
       <c r="M20" s="16"/>
     </row>
@@ -8326,19 +8326,19 @@
       <c r="M24" s="12"/>
     </row>
     <row r="25" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="492" t="s">
+      <c r="A25" s="489" t="s">
         <v>88</v>
       </c>
-      <c r="B25" s="493"/>
-      <c r="C25" s="493"/>
-      <c r="D25" s="493"/>
-      <c r="E25" s="493"/>
-      <c r="F25" s="493"/>
-      <c r="G25" s="493"/>
-      <c r="H25" s="493"/>
-      <c r="I25" s="493"/>
-      <c r="J25" s="493"/>
-      <c r="K25" s="494"/>
+      <c r="B25" s="490"/>
+      <c r="C25" s="490"/>
+      <c r="D25" s="490"/>
+      <c r="E25" s="490"/>
+      <c r="F25" s="490"/>
+      <c r="G25" s="490"/>
+      <c r="H25" s="490"/>
+      <c r="I25" s="490"/>
+      <c r="J25" s="490"/>
+      <c r="K25" s="491"/>
       <c r="L25" s="12"/>
       <c r="M25" s="12"/>
     </row>
@@ -8393,19 +8393,19 @@
       <c r="M28" s="12"/>
     </row>
     <row r="29" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="492" t="s">
+      <c r="A29" s="489" t="s">
         <v>86</v>
       </c>
-      <c r="B29" s="493"/>
-      <c r="C29" s="493"/>
-      <c r="D29" s="493"/>
-      <c r="E29" s="493"/>
-      <c r="F29" s="493"/>
-      <c r="G29" s="493"/>
-      <c r="H29" s="493"/>
-      <c r="I29" s="493"/>
-      <c r="J29" s="493"/>
-      <c r="K29" s="494"/>
+      <c r="B29" s="490"/>
+      <c r="C29" s="490"/>
+      <c r="D29" s="490"/>
+      <c r="E29" s="490"/>
+      <c r="F29" s="490"/>
+      <c r="G29" s="490"/>
+      <c r="H29" s="490"/>
+      <c r="I29" s="490"/>
+      <c r="J29" s="490"/>
+      <c r="K29" s="491"/>
       <c r="L29" s="12"/>
       <c r="M29" s="12"/>
     </row>
@@ -8500,19 +8500,19 @@
       <c r="M34" s="16"/>
     </row>
     <row r="35" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="492" t="s">
+      <c r="A35" s="489" t="s">
         <v>87</v>
       </c>
-      <c r="B35" s="493"/>
-      <c r="C35" s="493"/>
-      <c r="D35" s="493"/>
-      <c r="E35" s="493"/>
-      <c r="F35" s="493"/>
-      <c r="G35" s="493"/>
-      <c r="H35" s="493"/>
-      <c r="I35" s="493"/>
-      <c r="J35" s="493"/>
-      <c r="K35" s="494"/>
+      <c r="B35" s="490"/>
+      <c r="C35" s="490"/>
+      <c r="D35" s="490"/>
+      <c r="E35" s="490"/>
+      <c r="F35" s="490"/>
+      <c r="G35" s="490"/>
+      <c r="H35" s="490"/>
+      <c r="I35" s="490"/>
+      <c r="J35" s="490"/>
+      <c r="K35" s="491"/>
       <c r="L35" s="20"/>
       <c r="M35" s="16"/>
     </row>
@@ -8604,57 +8604,57 @@
       <c r="P40"/>
     </row>
     <row r="41" spans="1:16" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="481" t="s">
+      <c r="A41" s="493" t="s">
         <v>218</v>
       </c>
-      <c r="B41" s="481"/>
-      <c r="C41" s="481"/>
-      <c r="D41" s="481"/>
-      <c r="E41" s="481"/>
-      <c r="F41" s="481"/>
-      <c r="G41" s="481"/>
-      <c r="H41" s="481"/>
-      <c r="I41" s="481"/>
-      <c r="J41" s="481"/>
-      <c r="K41" s="481"/>
+      <c r="B41" s="493"/>
+      <c r="C41" s="493"/>
+      <c r="D41" s="493"/>
+      <c r="E41" s="493"/>
+      <c r="F41" s="493"/>
+      <c r="G41" s="493"/>
+      <c r="H41" s="493"/>
+      <c r="I41" s="493"/>
+      <c r="J41" s="493"/>
+      <c r="K41" s="493"/>
       <c r="M41" s="12"/>
       <c r="N41"/>
       <c r="O41"/>
       <c r="P41"/>
     </row>
     <row r="42" spans="1:16" ht="39.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="482" t="s">
+      <c r="A42" s="488" t="s">
         <v>219</v>
       </c>
-      <c r="B42" s="482"/>
-      <c r="C42" s="482"/>
-      <c r="D42" s="482"/>
-      <c r="E42" s="482"/>
-      <c r="F42" s="482"/>
-      <c r="G42" s="482"/>
-      <c r="H42" s="482"/>
-      <c r="I42" s="482"/>
-      <c r="J42" s="482"/>
-      <c r="K42" s="482"/>
+      <c r="B42" s="488"/>
+      <c r="C42" s="488"/>
+      <c r="D42" s="488"/>
+      <c r="E42" s="488"/>
+      <c r="F42" s="488"/>
+      <c r="G42" s="488"/>
+      <c r="H42" s="488"/>
+      <c r="I42" s="488"/>
+      <c r="J42" s="488"/>
+      <c r="K42" s="488"/>
       <c r="M42" s="12"/>
       <c r="N42"/>
       <c r="O42"/>
       <c r="P42"/>
     </row>
     <row r="43" spans="1:16" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="482" t="s">
+      <c r="A43" s="488" t="s">
         <v>220</v>
       </c>
-      <c r="B43" s="482"/>
-      <c r="C43" s="482"/>
-      <c r="D43" s="482"/>
-      <c r="E43" s="482"/>
-      <c r="F43" s="482"/>
-      <c r="G43" s="482"/>
-      <c r="H43" s="482"/>
-      <c r="I43" s="482"/>
-      <c r="J43" s="482"/>
-      <c r="K43" s="482"/>
+      <c r="B43" s="488"/>
+      <c r="C43" s="488"/>
+      <c r="D43" s="488"/>
+      <c r="E43" s="488"/>
+      <c r="F43" s="488"/>
+      <c r="G43" s="488"/>
+      <c r="H43" s="488"/>
+      <c r="I43" s="488"/>
+      <c r="J43" s="488"/>
+      <c r="K43" s="488"/>
       <c r="L43" s="134"/>
       <c r="M43" s="12"/>
       <c r="N43"/>
@@ -8662,19 +8662,19 @@
       <c r="P43"/>
     </row>
     <row r="44" spans="1:16" ht="27.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="482" t="s">
+      <c r="A44" s="488" t="s">
         <v>221</v>
       </c>
-      <c r="B44" s="482"/>
-      <c r="C44" s="482"/>
-      <c r="D44" s="482"/>
-      <c r="E44" s="482"/>
-      <c r="F44" s="482"/>
-      <c r="G44" s="482"/>
-      <c r="H44" s="482"/>
-      <c r="I44" s="482"/>
-      <c r="J44" s="482"/>
-      <c r="K44" s="482"/>
+      <c r="B44" s="488"/>
+      <c r="C44" s="488"/>
+      <c r="D44" s="488"/>
+      <c r="E44" s="488"/>
+      <c r="F44" s="488"/>
+      <c r="G44" s="488"/>
+      <c r="H44" s="488"/>
+      <c r="I44" s="488"/>
+      <c r="J44" s="488"/>
+      <c r="K44" s="488"/>
       <c r="L44" s="132"/>
       <c r="M44" s="12"/>
       <c r="N44"/>
@@ -8682,19 +8682,19 @@
       <c r="P44"/>
     </row>
     <row r="45" spans="1:16" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="483" t="s">
+      <c r="A45" s="494" t="s">
         <v>222</v>
       </c>
-      <c r="B45" s="483"/>
-      <c r="C45" s="483"/>
-      <c r="D45" s="483"/>
-      <c r="E45" s="483"/>
-      <c r="F45" s="483"/>
-      <c r="G45" s="483"/>
-      <c r="H45" s="483"/>
-      <c r="I45" s="483"/>
-      <c r="J45" s="483"/>
-      <c r="K45" s="483"/>
+      <c r="B45" s="494"/>
+      <c r="C45" s="494"/>
+      <c r="D45" s="494"/>
+      <c r="E45" s="494"/>
+      <c r="F45" s="494"/>
+      <c r="G45" s="494"/>
+      <c r="H45" s="494"/>
+      <c r="I45" s="494"/>
+      <c r="J45" s="494"/>
+      <c r="K45" s="494"/>
       <c r="L45" s="319"/>
       <c r="M45" s="319"/>
       <c r="N45" s="319"/>
@@ -8702,17 +8702,17 @@
       <c r="P45"/>
     </row>
     <row r="46" spans="1:16" ht="3.6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="436"/>
-      <c r="B46" s="436"/>
-      <c r="C46" s="436"/>
-      <c r="D46" s="436"/>
-      <c r="E46" s="436"/>
-      <c r="F46" s="436"/>
-      <c r="G46" s="436"/>
-      <c r="H46" s="436"/>
-      <c r="I46" s="436"/>
-      <c r="J46" s="436"/>
-      <c r="K46" s="436"/>
+      <c r="A46" s="435"/>
+      <c r="B46" s="435"/>
+      <c r="C46" s="435"/>
+      <c r="D46" s="435"/>
+      <c r="E46" s="435"/>
+      <c r="F46" s="435"/>
+      <c r="G46" s="435"/>
+      <c r="H46" s="435"/>
+      <c r="I46" s="435"/>
+      <c r="J46" s="435"/>
+      <c r="K46" s="435"/>
       <c r="L46" s="319"/>
       <c r="M46" s="319"/>
       <c r="N46" s="319"/>
@@ -8893,9 +8893,6 @@
     <protectedRange sqref="D5:D6" name="Rango3_3_1_1_1_1_1_2_1_1_1"/>
   </protectedRanges>
   <mergeCells count="17">
-    <mergeCell ref="C8:H8"/>
-    <mergeCell ref="A41:K41"/>
-    <mergeCell ref="A42:K42"/>
     <mergeCell ref="A44:K44"/>
     <mergeCell ref="A45:K45"/>
     <mergeCell ref="A2:K2"/>
@@ -8910,6 +8907,9 @@
     <mergeCell ref="C5:H5"/>
     <mergeCell ref="C6:H6"/>
     <mergeCell ref="C7:H7"/>
+    <mergeCell ref="C8:H8"/>
+    <mergeCell ref="A41:K41"/>
+    <mergeCell ref="A42:K42"/>
   </mergeCells>
   <phoneticPr fontId="5" type="noConversion"/>
   <dataValidations count="1">
@@ -8947,25 +8947,25 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="18" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B1" s="497" t="s">
+      <c r="B1" s="496" t="s">
         <v>148</v>
       </c>
-      <c r="C1" s="497"/>
-      <c r="D1" s="497"/>
-      <c r="E1" s="497"/>
-      <c r="F1" s="497"/>
-      <c r="G1" s="497"/>
-      <c r="H1" s="497"/>
-      <c r="I1" s="497"/>
+      <c r="C1" s="496"/>
+      <c r="D1" s="496"/>
+      <c r="E1" s="496"/>
+      <c r="F1" s="496"/>
+      <c r="G1" s="496"/>
+      <c r="H1" s="496"/>
+      <c r="I1" s="496"/>
     </row>
     <row r="2" spans="1:14" ht="4.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="3" spans="1:14" ht="11.4" x14ac:dyDescent="0.2">
-      <c r="B3" s="496" t="s">
+      <c r="B3" s="495" t="s">
         <v>100</v>
       </c>
-      <c r="C3" s="496"/>
-      <c r="D3" s="496"/>
-      <c r="E3" s="496"/>
+      <c r="C3" s="495"/>
+      <c r="D3" s="495"/>
+      <c r="E3" s="495"/>
       <c r="F3" s="184"/>
       <c r="G3" s="249" t="s">
         <v>105</v>
@@ -9056,10 +9056,10 @@
       <c r="G8" s="212" t="s">
         <v>115</v>
       </c>
-      <c r="J8" s="503" t="s">
+      <c r="J8" s="502" t="s">
         <v>136</v>
       </c>
-      <c r="K8" s="504"/>
+      <c r="K8" s="503"/>
       <c r="N8" s="183"/>
     </row>
     <row r="9" spans="1:14" ht="21.6" customHeight="1" x14ac:dyDescent="0.2">
@@ -9123,15 +9123,15 @@
     </row>
     <row r="12" spans="1:14" ht="24.6" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="126"/>
-      <c r="B12" s="502" t="s">
+      <c r="B12" s="501" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="502"/>
-      <c r="D12" s="502"/>
-      <c r="E12" s="502"/>
-      <c r="F12" s="502"/>
-      <c r="G12" s="502"/>
-      <c r="H12" s="502"/>
+      <c r="C12" s="501"/>
+      <c r="D12" s="501"/>
+      <c r="E12" s="501"/>
+      <c r="F12" s="501"/>
+      <c r="G12" s="501"/>
+      <c r="H12" s="501"/>
       <c r="J12" s="304" t="s">
         <v>139</v>
       </c>
@@ -9369,12 +9369,12 @@
     </row>
     <row r="23" spans="1:12" ht="27" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="20"/>
-      <c r="B23" s="498" t="s">
+      <c r="B23" s="497" t="s">
         <v>60</v>
       </c>
-      <c r="C23" s="499"/>
-      <c r="D23" s="499"/>
-      <c r="E23" s="499"/>
+      <c r="C23" s="498"/>
+      <c r="D23" s="498"/>
+      <c r="E23" s="498"/>
       <c r="F23" s="204" t="s">
         <v>63</v>
       </c>
@@ -9394,10 +9394,10 @@
       </c>
     </row>
     <row r="24" spans="1:12" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B24" s="500"/>
-      <c r="C24" s="501"/>
-      <c r="D24" s="501"/>
-      <c r="E24" s="501"/>
+      <c r="B24" s="499"/>
+      <c r="C24" s="500"/>
+      <c r="D24" s="500"/>
+      <c r="E24" s="500"/>
       <c r="F24" s="207" t="s">
         <v>118</v>
       </c>
@@ -9961,16 +9961,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="505"/>
-      <c r="B1" s="506"/>
-      <c r="C1" s="511" t="s">
+      <c r="A1" s="504"/>
+      <c r="B1" s="505"/>
+      <c r="C1" s="510" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="512"/>
-      <c r="E1" s="512"/>
-      <c r="F1" s="512"/>
-      <c r="G1" s="512"/>
-      <c r="H1" s="513"/>
+      <c r="D1" s="511"/>
+      <c r="E1" s="511"/>
+      <c r="F1" s="511"/>
+      <c r="G1" s="511"/>
+      <c r="H1" s="512"/>
       <c r="I1" s="22" t="s">
         <v>9</v>
       </c>
@@ -9979,14 +9979,14 @@
       </c>
     </row>
     <row r="2" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="507"/>
-      <c r="B2" s="508"/>
-      <c r="C2" s="514"/>
-      <c r="D2" s="515"/>
-      <c r="E2" s="515"/>
-      <c r="F2" s="515"/>
-      <c r="G2" s="515"/>
-      <c r="H2" s="516"/>
+      <c r="A2" s="506"/>
+      <c r="B2" s="507"/>
+      <c r="C2" s="513"/>
+      <c r="D2" s="514"/>
+      <c r="E2" s="514"/>
+      <c r="F2" s="514"/>
+      <c r="G2" s="514"/>
+      <c r="H2" s="515"/>
       <c r="I2" s="22" t="s">
         <v>11</v>
       </c>
@@ -9995,30 +9995,30 @@
       </c>
     </row>
     <row r="3" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="507"/>
-      <c r="B3" s="508"/>
-      <c r="C3" s="514"/>
-      <c r="D3" s="515"/>
-      <c r="E3" s="515"/>
-      <c r="F3" s="515"/>
-      <c r="G3" s="515"/>
-      <c r="H3" s="516"/>
+      <c r="A3" s="506"/>
+      <c r="B3" s="507"/>
+      <c r="C3" s="513"/>
+      <c r="D3" s="514"/>
+      <c r="E3" s="514"/>
+      <c r="F3" s="514"/>
+      <c r="G3" s="514"/>
+      <c r="H3" s="515"/>
       <c r="I3" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="J3" s="432">
+      <c r="J3" s="431">
         <v>46146</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="509"/>
-      <c r="B4" s="510"/>
-      <c r="C4" s="517"/>
-      <c r="D4" s="518"/>
-      <c r="E4" s="518"/>
-      <c r="F4" s="518"/>
-      <c r="G4" s="518"/>
-      <c r="H4" s="519"/>
+      <c r="A4" s="508"/>
+      <c r="B4" s="509"/>
+      <c r="C4" s="516"/>
+      <c r="D4" s="517"/>
+      <c r="E4" s="517"/>
+      <c r="F4" s="517"/>
+      <c r="G4" s="517"/>
+      <c r="H4" s="518"/>
       <c r="I4" s="22" t="s">
         <v>13</v>
       </c>
@@ -10030,17 +10030,17 @@
       <c r="A6" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="520" t="s">
+      <c r="B6" s="519" t="s">
         <v>144</v>
       </c>
-      <c r="C6" s="521"/>
-      <c r="D6" s="521"/>
-      <c r="E6" s="521"/>
-      <c r="F6" s="521"/>
-      <c r="G6" s="521"/>
-      <c r="H6" s="521"/>
-      <c r="I6" s="521"/>
-      <c r="J6" s="522"/>
+      <c r="C6" s="520"/>
+      <c r="D6" s="520"/>
+      <c r="E6" s="520"/>
+      <c r="F6" s="520"/>
+      <c r="G6" s="520"/>
+      <c r="H6" s="520"/>
+      <c r="I6" s="520"/>
+      <c r="J6" s="521"/>
     </row>
     <row r="7" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="25" t="s">
@@ -10320,10 +10320,10 @@
         <v>31</v>
       </c>
       <c r="I26" s="50"/>
-      <c r="J26" s="523" t="s">
+      <c r="J26" s="522" t="s">
         <v>34</v>
       </c>
-      <c r="K26" s="523"/>
+      <c r="K26" s="522"/>
       <c r="L26" s="284" t="s">
         <v>35</v>
       </c>
@@ -10374,11 +10374,11 @@
       <c r="I27" s="303" t="s">
         <v>125</v>
       </c>
-      <c r="J27" s="526" t="str">
+      <c r="J27" s="525" t="str">
         <f>+A27</f>
         <v xml:space="preserve">Masa de la muestra &gt; 3/8 (g), </v>
       </c>
-      <c r="K27" s="527"/>
+      <c r="K27" s="526"/>
       <c r="L27" s="282">
         <f>+H27</f>
         <v>0</v>
@@ -10427,11 +10427,11 @@
         <v>31</v>
       </c>
       <c r="I28" s="50"/>
-      <c r="J28" s="528" t="str">
+      <c r="J28" s="527" t="str">
         <f>+A31</f>
         <v xml:space="preserve">Masa de la muestra &lt; 3/8 (g), </v>
       </c>
-      <c r="K28" s="529"/>
+      <c r="K28" s="528"/>
       <c r="L28" s="283">
         <f>+H31</f>
         <v>0</v>
@@ -10480,11 +10480,11 @@
         <v>31</v>
       </c>
       <c r="I29" s="50"/>
-      <c r="J29" s="530" t="str">
+      <c r="J29" s="529" t="str">
         <f>+A36</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K29" s="531"/>
+      <c r="K29" s="530"/>
       <c r="L29" s="283" t="e">
         <f>+H36</f>
         <v>#DIV/0!</v>
@@ -10533,11 +10533,11 @@
         <v>31</v>
       </c>
       <c r="I30" s="50"/>
-      <c r="J30" s="532" t="str">
+      <c r="J30" s="531" t="str">
         <f>+A40</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K30" s="533"/>
+      <c r="K30" s="532"/>
       <c r="L30" s="283" t="e">
         <f>+H40</f>
         <v>#DIV/0!</v>
@@ -10590,11 +10590,11 @@
       <c r="I31" s="303" t="s">
         <v>126</v>
       </c>
-      <c r="J31" s="528" t="str">
+      <c r="J31" s="527" t="str">
         <f>+A45</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K31" s="529"/>
+      <c r="K31" s="528"/>
       <c r="L31" s="283">
         <f>+H45</f>
         <v>0</v>
@@ -10643,11 +10643,11 @@
         <v>31</v>
       </c>
       <c r="I32" s="50"/>
-      <c r="J32" s="534" t="str">
+      <c r="J32" s="533" t="str">
         <f>+A49</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K32" s="535"/>
+      <c r="K32" s="534"/>
       <c r="L32" s="283">
         <f>+H49</f>
         <v>0</v>
@@ -10696,11 +10696,11 @@
         <v>31</v>
       </c>
       <c r="I33" s="50"/>
-      <c r="J33" s="524" t="str">
+      <c r="J33" s="523" t="str">
         <f>+A53</f>
         <v xml:space="preserve">factor de presición </v>
       </c>
-      <c r="K33" s="525"/>
+      <c r="K33" s="524"/>
       <c r="L33" s="283">
         <f>+H53</f>
         <v>0.1709624577086255</v>
@@ -11728,10 +11728,10 @@
         <v>31</v>
       </c>
       <c r="I58" s="50"/>
-      <c r="J58" s="523" t="s">
+      <c r="J58" s="522" t="s">
         <v>34</v>
       </c>
-      <c r="K58" s="523"/>
+      <c r="K58" s="522"/>
       <c r="L58" s="284" t="s">
         <v>35</v>
       </c>
@@ -11780,11 +11780,11 @@
       <c r="I59" s="303" t="s">
         <v>125</v>
       </c>
-      <c r="J59" s="536" t="str">
+      <c r="J59" s="535" t="str">
         <f>+A59</f>
         <v xml:space="preserve">Masa de la muestra &gt; 3/8 (g), </v>
       </c>
-      <c r="K59" s="527"/>
+      <c r="K59" s="526"/>
       <c r="L59" s="282">
         <f>+H59</f>
         <v>0</v>
@@ -11831,11 +11831,11 @@
         <v>31</v>
       </c>
       <c r="I60" s="50"/>
-      <c r="J60" s="528" t="str">
+      <c r="J60" s="527" t="str">
         <f>+A63</f>
         <v xml:space="preserve">Masa de la muestra &lt; 3/8 (g), </v>
       </c>
-      <c r="K60" s="529"/>
+      <c r="K60" s="528"/>
       <c r="L60" s="283">
         <f>+H63</f>
         <v>0</v>
@@ -11882,11 +11882,11 @@
         <v>31</v>
       </c>
       <c r="I61" s="50"/>
-      <c r="J61" s="530" t="str">
+      <c r="J61" s="529" t="str">
         <f>+A68</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K61" s="531"/>
+      <c r="K61" s="530"/>
       <c r="L61" s="283" t="e">
         <f>+H68</f>
         <v>#DIV/0!</v>
@@ -11935,11 +11935,11 @@
         <v>31</v>
       </c>
       <c r="I62" s="50"/>
-      <c r="J62" s="532" t="str">
+      <c r="J62" s="531" t="str">
         <f>+A72</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K62" s="533"/>
+      <c r="K62" s="532"/>
       <c r="L62" s="283" t="e">
         <f>+H72</f>
         <v>#DIV/0!</v>
@@ -11992,11 +11992,11 @@
       <c r="I63" s="303" t="s">
         <v>126</v>
       </c>
-      <c r="J63" s="540" t="str">
+      <c r="J63" s="539" t="str">
         <f>+A77</f>
         <v>Masa particulas Fracturadas (g)</v>
       </c>
-      <c r="K63" s="529"/>
+      <c r="K63" s="528"/>
       <c r="L63" s="283">
         <f>+H77</f>
         <v>0</v>
@@ -12032,11 +12032,11 @@
         <v>31</v>
       </c>
       <c r="I64" s="50"/>
-      <c r="J64" s="534" t="str">
+      <c r="J64" s="533" t="str">
         <f>+A81</f>
         <v>Masa particulas que no cumplen el criterio especificado (g)</v>
       </c>
-      <c r="K64" s="535"/>
+      <c r="K64" s="534"/>
       <c r="L64" s="283">
         <f>+H81</f>
         <v>0</v>
@@ -12072,11 +12072,11 @@
         <v>31</v>
       </c>
       <c r="I65" s="50"/>
-      <c r="J65" s="524" t="str">
+      <c r="J65" s="523" t="str">
         <f>+A85</f>
         <v xml:space="preserve">factor de presición </v>
       </c>
-      <c r="K65" s="525"/>
+      <c r="K65" s="524"/>
       <c r="L65" s="283">
         <f>+H85</f>
         <v>0.15395666666666558</v>
@@ -12744,22 +12744,22 @@
       <c r="M87" s="45"/>
     </row>
     <row r="90" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A90" s="433" t="s">
+      <c r="A90" s="432" t="s">
         <v>209</v>
       </c>
-      <c r="B90" s="541" t="s">
+      <c r="B90" s="540" t="s">
         <v>210</v>
       </c>
-      <c r="C90" s="542"/>
-      <c r="D90" s="434"/>
-      <c r="E90" s="543" t="s">
+      <c r="C90" s="541"/>
+      <c r="D90" s="433"/>
+      <c r="E90" s="542" t="s">
         <v>211</v>
       </c>
-      <c r="F90" s="543"/>
-      <c r="G90" s="544" t="s">
+      <c r="F90" s="542"/>
+      <c r="G90" s="543" t="s">
         <v>212</v>
       </c>
-      <c r="H90" s="545"/>
+      <c r="H90" s="544"/>
     </row>
     <row r="91" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A91" s="32"/>
@@ -12772,22 +12772,22 @@
       <c r="H91" s="32"/>
     </row>
     <row r="92" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A92" s="435" t="s">
+      <c r="A92" s="434" t="s">
         <v>213</v>
       </c>
-      <c r="B92" s="537">
+      <c r="B92" s="536">
         <v>45604</v>
       </c>
-      <c r="C92" s="538"/>
+      <c r="C92" s="537"/>
       <c r="D92" s="32"/>
-      <c r="E92" s="539" t="s">
+      <c r="E92" s="538" t="s">
         <v>214</v>
       </c>
-      <c r="F92" s="539"/>
-      <c r="G92" s="537">
+      <c r="F92" s="538"/>
+      <c r="G92" s="536">
         <v>45605</v>
       </c>
-      <c r="H92" s="538"/>
+      <c r="H92" s="537"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="8bpvulMySDhbCinMJCKA6z/Rt8I37vsDQJVa4PyGNTLespzr8fQA8IH94JgjrRjZWt4j2jiXTM/mppn7uL1Pfg==" saltValue="zH87836e9WKbmOJcNpq46A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
@@ -12836,18 +12836,18 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="B2" s="546" t="s">
+      <c r="B2" s="545" t="s">
         <v>47</v>
       </c>
-      <c r="C2" s="546"/>
-      <c r="D2" s="546"/>
-      <c r="E2" s="546"/>
-      <c r="F2" s="546"/>
-      <c r="G2" s="546"/>
+      <c r="C2" s="545"/>
+      <c r="D2" s="545"/>
+      <c r="E2" s="545"/>
+      <c r="F2" s="545"/>
+      <c r="G2" s="545"/>
     </row>
     <row r="6" spans="2:10" x14ac:dyDescent="0.25">
-      <c r="I6" s="547"/>
-      <c r="J6" s="548"/>
+      <c r="I6" s="546"/>
+      <c r="J6" s="547"/>
     </row>
     <row r="7" spans="2:10" x14ac:dyDescent="0.25">
       <c r="B7" s="107" t="s">
@@ -13283,72 +13283,72 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="437"/>
+      <c r="A2" s="436"/>
     </row>
     <row r="3" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A3" s="438" t="s">
+      <c r="A3" s="437" t="s">
         <v>217</v>
       </c>
     </row>
     <row r="4" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A4" s="438" t="s">
+      <c r="A4" s="437" t="s">
         <v>54</v>
       </c>
-      <c r="B4" s="439">
+      <c r="B4" s="438">
         <v>45789</v>
       </c>
     </row>
     <row r="5" spans="1:10" ht="13.8" x14ac:dyDescent="0.25">
-      <c r="A5" s="438"/>
-      <c r="B5" s="440"/>
+      <c r="A5" s="437"/>
+      <c r="B5" s="439"/>
     </row>
     <row r="6" spans="1:10" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="437" t="s">
+      <c r="A6" s="436" t="s">
         <v>127</v>
       </c>
-      <c r="D6" s="437"/>
-      <c r="G6" s="437" t="s">
+      <c r="D6" s="436"/>
+      <c r="G6" s="436" t="s">
         <v>128</v>
       </c>
-      <c r="J6" s="437"/>
+      <c r="J6" s="436"/>
     </row>
     <row r="7" spans="1:10" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="123" t="s">
         <v>215</v>
       </c>
-      <c r="B7" s="555">
+      <c r="B7" s="554">
         <v>0.1709624577086255</v>
       </c>
-      <c r="C7" s="555"/>
-      <c r="D7" s="555"/>
-      <c r="E7" s="437"/>
+      <c r="C7" s="554"/>
+      <c r="D7" s="554"/>
+      <c r="E7" s="436"/>
       <c r="G7" s="123" t="s">
         <v>215</v>
       </c>
-      <c r="H7" s="549">
+      <c r="H7" s="548">
         <v>0.15395666666666558</v>
       </c>
-      <c r="I7" s="550"/>
-      <c r="J7" s="551"/>
+      <c r="I7" s="549"/>
+      <c r="J7" s="550"/>
     </row>
     <row r="8" spans="1:10" ht="23.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="123" t="s">
         <v>216</v>
       </c>
-      <c r="B8" s="556">
+      <c r="B8" s="555">
         <v>2.4584592209305228E-2</v>
       </c>
-      <c r="C8" s="556"/>
-      <c r="D8" s="556"/>
-      <c r="E8" s="437"/>
+      <c r="C8" s="555"/>
+      <c r="D8" s="555"/>
+      <c r="E8" s="436"/>
       <c r="G8" s="123" t="s">
         <v>216</v>
       </c>
-      <c r="H8" s="552">
+      <c r="H8" s="551">
         <v>2.3680740741075144E-2</v>
       </c>
-      <c r="I8" s="553"/>
-      <c r="J8" s="554"/>
+      <c r="I8" s="552"/>
+      <c r="J8" s="553"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="flW1XesbHlqTRTFELima/nxFJyeWIMi6FUGaLJDC0/kTtqlexRtX9Ql60qMdhZ24V0IUD+HXrOilxh83xKkl4Q==" saltValue="sXC/B0cfAHOFWzklDbqUSA==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>

</xml_diff>